<commit_message>
RTM v02: aponta para a especificação de requisitos v02 e deixa de usar o Backlog v03 como fonte
A baseline passa a citar a Especificação de Requisitos v02 e a Documentação da Arquitetura v02 (rascunhos)
e o Backlog v02 assinado; a proposta de Backlog v03 ainda não está aprovada.
As lacunas L5, L6 e L9 refletem o estado atual dos rascunhos.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FJ4FqWF1hX4FXNtdipqpfU
</commit_message>
<xml_diff>
--- a/04-artefactos-tecnicos/04.03-requisitos-e-rtm/m3-requirements-traceability-matrix-v02.xlsx
+++ b/04-artefactos-tecnicos/04.03-requisitos-e-rtm/m3-requirements-traceability-matrix-v02.xlsx
@@ -1029,7 +1029,7 @@
       <c r="C4" s="30" t="n"/>
       <c r="D4" s="11" t="inlineStr">
         <is>
-          <t>m2-especificacao-requisitos-v01.md</t>
+          <t>m3-especificacao-requisitos-v02.md (rascunho, PR #179); a v01 (m2-especificacao-requisitos-v01.md) mantém-se como histórico</t>
         </is>
       </c>
       <c r="E4" s="31" t="n"/>
@@ -1063,7 +1063,7 @@
       <c r="K5" s="31" t="n"/>
       <c r="L5" s="32" t="n"/>
     </row>
-    <row r="6" ht="32.25" customHeight="1">
+    <row r="6" ht="48" customHeight="1">
       <c r="A6" s="10" t="inlineStr">
         <is>
           <t>Baseline considerada na m3</t>
@@ -1073,7 +1073,7 @@
       <c r="C6" s="30" t="n"/>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>Declaração de Âmbito v05; Documentação da API v02 (37 endpoints); Especificações dos Casos de Uso v02; Modelos de Classes v02; Plano de Testes do Backend v02; Backlog de Projeto v03 (rascunho)</t>
+          <t>Declaração de Âmbito v05; Especificação de Requisitos v02 (rascunho); Documentação da API v02 (37 endpoints); Especificações dos Casos de Uso v02; Modelos de Classes v02; Documentação da Arquitetura v02 (rascunho); Plano de Testes do Backend v02; Backlog de Projeto v02 (assinado). A proposta de Backlog v03 ainda não foi aprovada e não serve de fonte.</t>
         </is>
       </c>
       <c r="E6" s="31" t="n"/>
@@ -5359,7 +5359,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="78.5" customHeight="1">
+    <row r="10" ht="107.5" customHeight="1">
       <c r="A10" s="40" t="n">
         <v>1</v>
       </c>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="F10" s="41" t="inlineStr">
         <is>
-          <t>Declaração de Âmbito v05; Documentação da API v02, secção 11; Backlog v03 (Issues I079–I081, I083–I085, I117, I119 e I124 descontinuadas). A RTM v01 prevê a conservação dos requisitos descontinuados.</t>
+          <t>Declaração de Âmbito v05; Especificação de Requisitos v02 (rascunho); Documentação da API v02, secção 11. As Issues I079–I081, I083–I085, I117, I119 e I124 constam do Backlog v02 assinado e a proposta de Backlog v03 (por aprovar) descontinua-as. A RTM v01 prevê a conservação dos requisitos descontinuados.</t>
         </is>
       </c>
     </row>
@@ -5415,7 +5415,7 @@
       </c>
       <c r="F11" s="41" t="inlineStr">
         <is>
-          <t>Backlog de Projeto v03 (rascunho): títulos das Issues I063–I078, I082, I086–I100, I108–I118, I121–I123, I129–I131 e I137.</t>
+          <t>Backlog de Projeto v02 (assinado): títulos das Issues I063–I078, I082, I086–I100, I108–I118, I121–I123, I129–I131 e I137.</t>
         </is>
       </c>
     </row>
@@ -5625,7 +5625,7 @@
       </c>
       <c r="F18" s="41" t="inlineStr">
         <is>
-          <t>Backlog v03 (rascunho) e Plano de Testes do Backend v02.</t>
+          <t>Backlog v02 (assinado) e Plano de Testes do Backend v02.</t>
         </is>
       </c>
     </row>
@@ -5727,7 +5727,7 @@
     <row r="27" ht="32" customHeight="1">
       <c r="A27" s="42" t="inlineStr">
         <is>
-          <t>As referências requisito → Issue foram lidas dos títulos do Backlog v03 (rascunho): se o Backlog Refinement mudar uma Issue, a linha correspondente deve ser atualizada.</t>
+          <t>As referências requisito → Issue foram lidas dos títulos das Issues do Backlog v02 (assinado): se o Backlog Refinement mudar uma Issue, a linha correspondente deve ser atualizada.</t>
         </is>
       </c>
     </row>
@@ -5940,7 +5940,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="93" customHeight="1">
+    <row r="9" ht="107.5" customHeight="1">
       <c r="A9" s="40" t="inlineStr">
         <is>
           <t>L5</t>
@@ -5958,7 +5958,7 @@
       </c>
       <c r="D9" s="41" t="inlineStr">
         <is>
-          <t>Os requisitos aparecem nas Issues do Backlog v03 (rascunho), mas não constam da Especificação de Requisitos v01 nem da API v02. Não se criaram linhas para não registar requisitos por aprovar. A Issue I024 cita uma «Especificação de Requisitos v02» que ainda não existe.</t>
+          <t>Os requisitos só aparecem na proposta de Backlog v03 (por aprovar). Não constam da Especificação de Requisitos v01, nem da v02 (rascunho, PR #179), nem da API v02. Não se criaram linhas para não registar requisitos por aprovar. A Issue I024 cita uma «Especificação de Requisitos v02», que existe agora em rascunho e sem esses requisitos.</t>
         </is>
       </c>
       <c r="E9" s="41" t="inlineStr">
@@ -5968,11 +5968,11 @@
       </c>
       <c r="F9" s="41" t="inlineStr">
         <is>
-          <t>Acrescentar as linhas quando a Especificação de Requisitos v02 estiver aprovada</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="78.5" customHeight="1">
+          <t>Acrescentar as linhas quando uma especificação de requisitos aprovada os definir</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="107.5" customHeight="1">
       <c r="A10" s="40" t="inlineStr">
         <is>
           <t>L6</t>
@@ -5985,12 +5985,12 @@
       </c>
       <c r="C10" s="41" t="inlineStr">
         <is>
-          <t>A Arquitetura continua na v01.</t>
+          <t>A Arquitetura v02 está em rascunho.</t>
         </is>
       </c>
       <c r="D10" s="41" t="inlineStr">
         <is>
-          <t>A Documentação da Arquitetura v01 ainda lista ARC-F005 e ARC-F007 e as tecnologias anteriores (por exemplo, Flutter). Os identificadores ARC mantêm-se; retiraram-se apenas ARC-F005 e ARC-F007 das linhas dos requisitos não funcionais.</t>
+          <t>A Documentação da Arquitetura v02 (rascunho, PR #181) retira ARC-F005 e ARC-F007 e atualiza as tecnologias. Os identificadores ARC dos módulos em âmbito mantêm-se, por isso esta RTM serve às duas versões. Enquanto a v02 não for aprovada, a v01 (que ainda lista ARC-F005, ARC-F007 e Flutter) é a versão entregue.</t>
         </is>
       </c>
       <c r="E10" s="41" t="inlineStr">
@@ -6000,7 +6000,7 @@
       </c>
       <c r="F10" s="41" t="inlineStr">
         <is>
-          <t>Atualizar quando existir a Arquitetura v02</t>
+          <t>Confirmar quando a Arquitetura v02 for aprovada</t>
         </is>
       </c>
     </row>
@@ -6081,12 +6081,12 @@
       </c>
       <c r="C13" s="41" t="inlineStr">
         <is>
-          <t>A Especificação de Requisitos v01 e outros documentos ainda tratam estes requisitos como ativos.</t>
+          <t>A Especificação de Requisitos v01 e outros documentos da m2 ainda tratam estes requisitos como ativos.</t>
         </is>
       </c>
       <c r="D13" s="41" t="inlineStr">
         <is>
-          <t>A decisão de âmbito consta da Declaração de Âmbito v05. A RTM regista-os como «7 - Descontinuado»; a Especificação de Requisitos v01 não foi alterada.</t>
+          <t>A decisão de âmbito consta da Declaração de Âmbito v05. A RTM regista-os como «7 - Descontinuado», tal como a Especificação de Requisitos v02 (rascunho, PR #179).</t>
         </is>
       </c>
       <c r="E13" s="41" t="inlineStr">
@@ -6096,7 +6096,7 @@
       </c>
       <c r="F13" s="41" t="inlineStr">
         <is>
-          <t>Alinhar na Especificação de Requisitos v02</t>
+          <t>Aprovar a Especificação de Requisitos v02</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
RTM v02: Issues de F005 e F007 passam a «a descontinuar no Backlog Refinement (por decidir)»
A proposta de Backlog v03 ainda não foi aprovada, por isso a RTM não afirma que as Issues já foram descontinuadas.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FJ4FqWF1hX4FXNtdipqpfU
</commit_message>
<xml_diff>
--- a/04-artefactos-tecnicos/04.03-requisitos-e-rtm/m3-requirements-traceability-matrix-v02.xlsx
+++ b/04-artefactos-tecnicos/04.03-requisitos-e-rtm/m3-requirements-traceability-matrix-v02.xlsx
@@ -3622,7 +3622,7 @@
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>Descontinuado — Issues descontinuadas: I079; I080; I081 (backend); I117 (web)</t>
+          <t>Descontinuado — Issues a descontinuar no Backlog Refinement (por decidir): I079; I080; I081 (backend); I117 (web)</t>
         </is>
       </c>
       <c r="G45" s="3" t="inlineStr">
@@ -3687,7 +3687,7 @@
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>Descontinuado — Issues descontinuadas: I079; I080; I081 (backend); I117 (web)</t>
+          <t>Descontinuado — Issues a descontinuar no Backlog Refinement (por decidir): I079; I080; I081 (backend); I117 (web)</t>
         </is>
       </c>
       <c r="G46" s="3" t="inlineStr">
@@ -3752,7 +3752,7 @@
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>Descontinuado — Issues descontinuadas: I079; I080; I081 (backend); I117 (web)</t>
+          <t>Descontinuado — Issues a descontinuar no Backlog Refinement (por decidir): I079; I080; I081 (backend); I117 (web)</t>
         </is>
       </c>
       <c r="G47" s="3" t="inlineStr">
@@ -3817,7 +3817,7 @@
       </c>
       <c r="F48" s="3" t="inlineStr">
         <is>
-          <t>Descontinuado — Issues descontinuadas: I079; I080; I081 (backend); I117 (web)</t>
+          <t>Descontinuado — Issues a descontinuar no Backlog Refinement (por decidir): I079; I080; I081 (backend); I117 (web)</t>
         </is>
       </c>
       <c r="G48" s="3" t="inlineStr">
@@ -3882,7 +3882,7 @@
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>Descontinuado — Issues descontinuadas: I079; I080; I081 (backend); I117 (web)</t>
+          <t>Descontinuado — Issues a descontinuar no Backlog Refinement (por decidir): I079; I080; I081 (backend); I117 (web)</t>
         </is>
       </c>
       <c r="G49" s="3" t="inlineStr">
@@ -3947,7 +3947,7 @@
       </c>
       <c r="F50" s="3" t="inlineStr">
         <is>
-          <t>Descontinuado — Issue descontinuada: I124 (mobile)</t>
+          <t>Descontinuado — Issue a descontinuar no Backlog Refinement (por decidir): I124 (mobile)</t>
         </is>
       </c>
       <c r="G50" s="3" t="inlineStr">
@@ -4347,7 +4347,7 @@
       </c>
       <c r="F56" s="3" t="inlineStr">
         <is>
-          <t>Descontinuado — Issues descontinuadas: I083; I084; I085 (backend); I119 (web)</t>
+          <t>Descontinuado — Issues a descontinuar no Backlog Refinement (por decidir): I083; I084; I085 (backend); I119 (web)</t>
         </is>
       </c>
       <c r="G56" s="3" t="inlineStr">
@@ -4412,7 +4412,7 @@
       </c>
       <c r="F57" s="3" t="inlineStr">
         <is>
-          <t>Descontinuado — Issues descontinuadas: I083; I084; I085 (backend); I119 (web)</t>
+          <t>Descontinuado — Issues a descontinuar no Backlog Refinement (por decidir): I083; I084; I085 (backend); I119 (web)</t>
         </is>
       </c>
       <c r="G57" s="3" t="inlineStr">
@@ -4477,7 +4477,7 @@
       </c>
       <c r="F58" s="3" t="inlineStr">
         <is>
-          <t>Descontinuado — Issues descontinuadas: I083; I084; I085 (backend); I119 (web)</t>
+          <t>Descontinuado — Issues a descontinuar no Backlog Refinement (por decidir): I083; I084; I085 (backend); I119 (web)</t>
         </is>
       </c>
       <c r="G58" s="3" t="inlineStr">
@@ -4542,7 +4542,7 @@
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>Descontinuado — Issues descontinuadas: I083; I084; I085 (backend); I119 (web)</t>
+          <t>Descontinuado — Issues a descontinuar no Backlog Refinement (por decidir): I083; I084; I085 (backend); I119 (web)</t>
         </is>
       </c>
       <c r="G59" s="3" t="inlineStr">
@@ -4607,7 +4607,7 @@
       </c>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>Descontinuado — Issues descontinuadas: I083; I084; I085 (backend); I119 (web)</t>
+          <t>Descontinuado — Issues a descontinuar no Backlog Refinement (por decidir): I083; I084; I085 (backend); I119 (web)</t>
         </is>
       </c>
       <c r="G60" s="3" t="inlineStr">

</xml_diff>

<commit_message>
RTM v02: acrescenta as Issues que o Backlog v02 liga a cada requisito e os endpoints EP-004, EP-012 e EP-021
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FJ4FqWF1hX4FXNtdipqpfU
</commit_message>
<xml_diff>
--- a/04-artefactos-tecnicos/04.03-requisitos-e-rtm/m3-requirements-traceability-matrix-v02.xlsx
+++ b/04-artefactos-tecnicos/04.03-requisitos-e-rtm/m3-requirements-traceability-matrix-v02.xlsx
@@ -1612,7 +1612,7 @@
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Previsto em m3 — implementação: I065; testes: I086; I092; I098
+          <t>Previsto em m3 — implementação: I065; I066; testes: I086; I092; I098
 Previsto em m4 — implementação web: I109; testes de sistema: web I129</t>
         </is>
       </c>
@@ -1679,13 +1679,13 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>Previsto em m3 — implementação: I066; testes: I086; I092; I098
+          <t>Previsto em m3 — implementação: I065; I066; testes: I086; I092; I098
 Previsto em m4 — implementação web: I109; testes de sistema: web I129</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>Previsto em m3 — EP-006 POST /utilizadores; EP-007 PUT /utilizadores/{id}
+          <t>Previsto em m3 — EP-004 GET /utilizadores; EP-006 POST /utilizadores; EP-007 PUT /utilizadores/{id}
 Lacuna L1: por implementar em 23/10/2026 (ver folha «Lacunas»).</t>
         </is>
       </c>
@@ -1702,7 +1702,7 @@
       </c>
       <c r="J16" s="3" t="inlineStr">
         <is>
-          <t>Previsto em m3 — CT-F001-05; CT-F001-06; CT-F001-11 (Plano de Testes do Backend v02, secção 10); endpoints EP-006, EP-007 (secção 15.1) com testes unitários, de integração e pedidos Postman (I086; I092; I098)
+          <t>Previsto em m3 — CT-F001-05; CT-F001-06; CT-F001-11 (Plano de Testes do Backend v02, secção 10); endpoints EP-004, EP-006, EP-007 (secção 15.1) com testes unitários, de integração e pedidos Postman (I086; I092; I098)
 Previsto em m4 — testes de sistema Web
 Lacuna L2: sem testes executados em 23/10/2026 (ver folha «Lacunas»).</t>
         </is>
@@ -1718,7 +1718,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="107.5" customHeight="1">
+    <row r="17" ht="122" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
           <t>RF009</t>
@@ -1746,13 +1746,13 @@
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Previsto em m3 — implementação: I066; testes: I086; I092; I098
+          <t>Previsto em m3 — implementação: I065; I066; testes: I086; I092; I098
 Previsto em m4 — implementação web: I109; testes de sistema: web I129</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>Previsto em m3 — EP-008 PATCH /utilizadores/{id}/estado
+          <t>Previsto em m3 — EP-004 GET /utilizadores; EP-008 PATCH /utilizadores/{id}/estado
 Lacuna L1: por implementar em 23/10/2026 (ver folha «Lacunas»).</t>
         </is>
       </c>
@@ -1769,7 +1769,7 @@
       </c>
       <c r="J17" s="3" t="inlineStr">
         <is>
-          <t>Previsto em m3 — CT-F001-02; CT-F001-06; CT-F001-07 (Plano de Testes do Backend v02, secção 10); endpoints EP-008 (secção 15.1) com testes unitários, de integração e pedidos Postman (I086; I092; I098)
+          <t>Previsto em m3 — CT-F001-02; CT-F001-06; CT-F001-07 (Plano de Testes do Backend v02, secção 10); endpoints EP-004, EP-008 (secção 15.1) com testes unitários, de integração e pedidos Postman (I086; I092; I098)
 Previsto em m4 — testes de sistema Web
 Lacuna L2: sem testes executados em 23/10/2026 (ver folha «Lacunas»).</t>
         </is>
@@ -2282,13 +2282,13 @@
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>Previsto em m3 — implementação: I069; testes: I092; I098
+          <t>Previsto em m3 — implementação: I068; I069; testes: I092; I098
 Previsto em m4 — implementação web: I112; testes de sistema: web I129</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>Previsto em m3 — EP-011 GET /clientes; EP-015 GET /animais
+          <t>Previsto em m3 — EP-011 GET /clientes; EP-012 GET /clientes/{id}; EP-015 GET /animais
 Lacuna L1: por implementar em 23/10/2026 (ver folha «Lacunas»).</t>
         </is>
       </c>
@@ -2305,7 +2305,7 @@
       </c>
       <c r="J25" s="3" t="inlineStr">
         <is>
-          <t>Previsto em m3 — CT-F002-02 (Plano de Testes do Backend v02, secção 10); endpoints EP-011, EP-015 (secção 15.1) com testes de integração e pedidos Postman (I092; I098)
+          <t>Previsto em m3 — CT-F002-02 (Plano de Testes do Backend v02, secção 10); endpoints EP-011, EP-012, EP-015 (secção 15.1) com testes de integração e pedidos Postman (I092; I098)
 Previsto em m4 — testes de sistema Web
 Lacuna L2: sem testes executados em 23/10/2026 (ver folha «Lacunas»).</t>
         </is>
@@ -2416,7 +2416,7 @@
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>Previsto em m3 — implementação: I067; testes: I087; I093; I099
+          <t>Previsto em m3 — implementação: I067; I071; testes: I087; I093; I099
 Previsto em m4 — implementação web: I110; testes de sistema: web I129</t>
         </is>
       </c>
@@ -2550,13 +2550,13 @@
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>Previsto em m3 — implementação: I073; testes: I087; I093; I099
+          <t>Previsto em m3 — implementação: I071; I073; testes: I087; I093; I099
 Previsto em m4 — implementação web: I113; testes de sistema: web I130</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>Previsto em m3 — EP-025 POST /consultas
+          <t>Previsto em m3 — EP-021 GET /veterinarios; EP-025 POST /consultas
 Lacuna L1: por implementar em 23/10/2026 (ver folha «Lacunas»).</t>
         </is>
       </c>
@@ -2573,7 +2573,7 @@
       </c>
       <c r="J29" s="3" t="inlineStr">
         <is>
-          <t>Previsto em m3 — CT-F003-01 (Plano de Testes do Backend v02, secção 10); endpoints EP-025 (secção 15.1) com testes unitários, de integração e pedidos Postman (I087; I093; I099)
+          <t>Previsto em m3 — CT-F003-01 (Plano de Testes do Backend v02, secção 10); endpoints EP-021, EP-025 (secção 15.1) com testes unitários, de integração e pedidos Postman (I087; I093; I099)
 Previsto em m4 — testes de sistema Web
 Lacuna L2: sem testes executados em 23/10/2026 (ver folha «Lacunas»).</t>
         </is>
@@ -2885,7 +2885,7 @@
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>Previsto em m3 — implementação: I075; testes: I087; I093; I099
+          <t>Previsto em m3 — implementação: I069; I072; I075; testes: I087; I093; I099
 Previsto em m4 — implementação web: I114; testes de sistema: web I130</t>
         </is>
       </c>
@@ -5389,7 +5389,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="49.5" customHeight="1">
+    <row r="11" ht="93" customHeight="1">
       <c r="A11" s="40" t="n">
         <v>2</v>
       </c>
@@ -5415,11 +5415,11 @@
       </c>
       <c r="F11" s="41" t="inlineStr">
         <is>
-          <t>Backlog de Projeto v02 (assinado): títulos das Issues I063–I078, I082, I086–I100, I108–I118, I121–I123, I129–I131 e I137.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="49.5" customHeight="1">
+          <t>Backlog de Projeto v02 (assinado): títulos das Issues I063–I078, I082, I086–I100, I108–I118, I121–I123, I129–I131 e I137 e, para as Issues de backend, os requisitos que cada uma refere em «Normas, modelos e referências».</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="64" customHeight="1">
       <c r="A12" s="40" t="n">
         <v>3</v>
       </c>
@@ -5440,7 +5440,7 @@
       </c>
       <c r="E12" s="41" t="inlineStr">
         <is>
-          <t>Endpoints inalterados e acrescentada a referência à lacuna L1.</t>
+          <t>Endpoints inalterados, exceto EP-004 (RF008, RF009), EP-012 (RF017) e EP-021 (RF021), acrescentados como na secção 12.4 da API v02. Acrescentada a referência à lacuna L1.</t>
         </is>
       </c>
       <c r="F12" s="41" t="inlineStr">

</xml_diff>

<commit_message>
RTM v02: RF026 deixa de citar a I075 e RF017 passa a citar a I111 no frontend web, como no Backlog v02
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FJ4FqWF1hX4FXNtdipqpfU
</commit_message>
<xml_diff>
--- a/04-artefactos-tecnicos/04.03-requisitos-e-rtm/m3-requirements-traceability-matrix-v02.xlsx
+++ b/04-artefactos-tecnicos/04.03-requisitos-e-rtm/m3-requirements-traceability-matrix-v02.xlsx
@@ -2283,7 +2283,7 @@
       <c r="F25" s="3" t="inlineStr">
         <is>
           <t>Previsto em m3 — implementação: I068; I069; testes: I092; I098
-Previsto em m4 — implementação web: I112; testes de sistema: web I129</t>
+Previsto em m4 — implementação web: I111; I112; testes de sistema: web I129</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr">
@@ -2885,7 +2885,7 @@
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>Previsto em m3 — implementação: I069; I072; I075; testes: I087; I093; I099
+          <t>Previsto em m3 — implementação: I069; I072; testes: I087; I093; I099
 Previsto em m4 — implementação web: I114; testes de sistema: web I130</t>
         </is>
       </c>
@@ -5415,7 +5415,7 @@
       </c>
       <c r="F11" s="41" t="inlineStr">
         <is>
-          <t>Backlog de Projeto v02 (assinado): títulos das Issues I063–I078, I082, I086–I100, I108–I118, I121–I123, I129–I131 e I137 e, para as Issues de backend, os requisitos que cada uma refere em «Normas, modelos e referências».</t>
+          <t>Backlog de Projeto v02 (assinado): títulos das Issues I063–I078, I082, I086–I100, I108–I118, I121–I123, I129–I131 e I137 e, para as Issues de backend e de frontend web, os requisitos que cada uma refere em «Normas, modelos e referências».</t>
         </is>
       </c>
     </row>

</xml_diff>